<commit_message>
complete 6 error groups, 8 normalization categories and 3 advanced extension features
</commit_message>
<xml_diff>
--- a/sample-data/danh-muc-san-pham-chuan.xlsx
+++ b/sample-data/danh-muc-san-pham-chuan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Danh mục chuẩn" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -424,13 +424,13 @@
         <v>9786045678901</v>
       </c>
       <c r="C2" t="str">
-        <v>NXB Tổng Hợp TPHCM</v>
+        <v>NXB Trẻ</v>
       </c>
       <c r="D2" t="str">
         <v>Kỹ năng sống</v>
       </c>
-      <c r="E2">
-        <v>86000</v>
+      <c r="E2" t="str">
+        <v>86.000</v>
       </c>
     </row>
     <row r="3">
@@ -441,13 +441,13 @@
         <v>9786045678902</v>
       </c>
       <c r="C3" t="str">
-        <v>NXB Hội Nhà Văn</v>
+        <v>NXB Nhã Nam</v>
       </c>
       <c r="D3" t="str">
         <v>Văn học</v>
       </c>
-      <c r="E3">
-        <v>79000</v>
+      <c r="E3" t="str">
+        <v>79.000</v>
       </c>
     </row>
     <row r="4">
@@ -463,8 +463,8 @@
       <c r="D4" t="str">
         <v>Kỹ năng sống</v>
       </c>
-      <c r="E4">
-        <v>90000</v>
+      <c r="E4" t="str">
+        <v>90.000</v>
       </c>
     </row>
     <row r="5">
@@ -480,8 +480,8 @@
       <c r="D5" t="str">
         <v>Kỹ năng sống</v>
       </c>
-      <c r="E5">
-        <v>95000</v>
+      <c r="E5" t="str">
+        <v>95.000</v>
       </c>
     </row>
     <row r="6">
@@ -497,13 +497,13 @@
       <c r="D6" t="str">
         <v>Văn học</v>
       </c>
-      <c r="E6">
-        <v>125000</v>
+      <c r="E6" t="str">
+        <v>125.000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Mắt Biếc</v>
+        <v>Đời Thay Đổi Khi Chúng Ta Thay Đổi</v>
       </c>
       <c r="B7" t="str">
         <v>9786045678906</v>
@@ -512,49 +512,49 @@
         <v>NXB Trẻ</v>
       </c>
       <c r="D7" t="str">
-        <v>Văn học</v>
-      </c>
-      <c r="E7">
-        <v>110000</v>
+        <v>Kỹ năng sống</v>
+      </c>
+      <c r="E7" t="str">
+        <v>68.000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Khéo Ăn Nói Sẽ Có Được Thiên Hạ</v>
+        <v>Cha Giàu Cha Nghèo</v>
       </c>
       <c r="B8" t="str">
         <v>9786045678907</v>
       </c>
       <c r="C8" t="str">
-        <v>NXB Văn Học</v>
+        <v>NXB Trẻ</v>
       </c>
       <c r="D8" t="str">
-        <v>Kỹ năng sống</v>
-      </c>
-      <c r="E8">
-        <v>110000</v>
+        <v>Kinh doanh</v>
+      </c>
+      <c r="E8" t="str">
+        <v>115.000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Đời Thay Đổi Khi Chúng Ta Thay Đổi</v>
+        <v>Đọc Vị Bất Kỳ Ai</v>
       </c>
       <c r="B9" t="str">
         <v>9786045678908</v>
       </c>
       <c r="C9" t="str">
-        <v>NXB Trẻ</v>
+        <v>NXB Thế Giới</v>
       </c>
       <c r="D9" t="str">
         <v>Tâm lý học</v>
       </c>
-      <c r="E9">
-        <v>75000</v>
+      <c r="E9" t="str">
+        <v>89.000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Cha Giàu Cha Nghèo</v>
+        <v>Mắt Biếc</v>
       </c>
       <c r="B10" t="str">
         <v>9786045678909</v>
@@ -563,134 +563,134 @@
         <v>NXB Trẻ</v>
       </c>
       <c r="D10" t="str">
-        <v>Kinh tế</v>
-      </c>
-      <c r="E10">
-        <v>135000</v>
+        <v>Văn học</v>
+      </c>
+      <c r="E10" t="str">
+        <v>110.000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Tư Duy Nhanh Và Chậm</v>
+        <v>Số Đỏ</v>
       </c>
       <c r="B11" t="str">
         <v>9786045678910</v>
       </c>
       <c r="C11" t="str">
-        <v>NXB Thế Giới</v>
+        <v>NXB Văn Học</v>
       </c>
       <c r="D11" t="str">
-        <v>Tâm lý học</v>
-      </c>
-      <c r="E11">
-        <v>220000</v>
+        <v>Văn học</v>
+      </c>
+      <c r="E11" t="str">
+        <v>65.000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Người Giàu Có Nhất Thành Babylon</v>
+        <v>Tư Duy Nhanh Và Chậm</v>
       </c>
       <c r="B12" t="str">
         <v>9786045678911</v>
       </c>
       <c r="C12" t="str">
-        <v>NXB Lao Động</v>
+        <v>NXB Thế Giới</v>
       </c>
       <c r="D12" t="str">
-        <v>Kinh tế</v>
-      </c>
-      <c r="E12">
-        <v>98000</v>
+        <v>Tâm lý học</v>
+      </c>
+      <c r="E12" t="str">
+        <v>210.000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Sức Mạnh Của Hiện Tại</v>
+        <v>Khéo Ăn Nói Sẽ Có Được Thiên Hạ</v>
       </c>
       <c r="B13" t="str">
         <v>9786045678912</v>
       </c>
       <c r="C13" t="str">
-        <v>NXB Tổng Hợp TPHCM</v>
+        <v>NXB Văn Học</v>
       </c>
       <c r="D13" t="str">
-        <v>Tâm lý học</v>
-      </c>
-      <c r="E13">
-        <v>130000</v>
+        <v>Kỹ năng sống</v>
+      </c>
+      <c r="E13" t="str">
+        <v>118.000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Đi Tìm Lẽ Sống</v>
+        <v>Dế Mèn Phiêu Lưu Ký</v>
       </c>
       <c r="B14" t="str">
         <v>9786045678913</v>
       </c>
       <c r="C14" t="str">
-        <v>NXB Tổng Hợp TPHCM</v>
+        <v>NXB Kim Đồng</v>
       </c>
       <c r="D14" t="str">
-        <v>Tâm lý học</v>
-      </c>
-      <c r="E14">
-        <v>88000</v>
+        <v>Thiếu nhi</v>
+      </c>
+      <c r="E14" t="str">
+        <v>55.000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Đọc Vị Bất Kỳ Ai</v>
+        <v>Chiếc Thuyền Ngoài Xa</v>
       </c>
       <c r="B15" t="str">
         <v>9786045678914</v>
       </c>
       <c r="C15" t="str">
-        <v>NXB Thế Giới</v>
+        <v>NXB Văn Học</v>
       </c>
       <c r="D15" t="str">
-        <v>Tâm lý học</v>
-      </c>
-      <c r="E15">
-        <v>89000</v>
+        <v>Văn học</v>
+      </c>
+      <c r="E15" t="str">
+        <v>48.000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Lược Sử Loài Người</v>
+        <v>Tắt Đèn</v>
       </c>
       <c r="B16" t="str">
         <v>9786045678915</v>
       </c>
       <c r="C16" t="str">
-        <v>NXB Tri Thức</v>
+        <v>NXB Văn Học</v>
       </c>
       <c r="D16" t="str">
-        <v>Lịch sử</v>
-      </c>
-      <c r="E16">
-        <v>240000</v>
+        <v>Văn học</v>
+      </c>
+      <c r="E16" t="str">
+        <v>52.000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Hạt Giống Tâm Hồn</v>
+        <v>Lão Hạc</v>
       </c>
       <c r="B17" t="str">
         <v>9786045678916</v>
       </c>
       <c r="C17" t="str">
-        <v>NXB Tổng Hợp TPHCM</v>
+        <v>NXB Văn Học</v>
       </c>
       <c r="D17" t="str">
-        <v>Kỹ năng sống</v>
-      </c>
-      <c r="E17">
-        <v>68000</v>
+        <v>Văn học</v>
+      </c>
+      <c r="E17" t="str">
+        <v>45.000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Số Đỏ</v>
+        <v>Vợ Nhặt</v>
       </c>
       <c r="B18" t="str">
         <v>9786045678917</v>
@@ -701,47 +701,47 @@
       <c r="D18" t="str">
         <v>Văn học</v>
       </c>
-      <c r="E18">
-        <v>65000</v>
+      <c r="E18" t="str">
+        <v>42.000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Tắt Đèn</v>
+        <v>Hạt Giống Tâm Hồn</v>
       </c>
       <c r="B19" t="str">
         <v>9786045678918</v>
       </c>
       <c r="C19" t="str">
-        <v>NXB Kim Đồng</v>
+        <v>NXB Tổng Hợp TP.HCM</v>
       </c>
       <c r="D19" t="str">
-        <v>Văn học</v>
-      </c>
-      <c r="E19">
-        <v>55000</v>
+        <v>Tâm lý học</v>
+      </c>
+      <c r="E19" t="str">
+        <v>75.000</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Rừng Na Uy</v>
+        <v>Sức Mạnh Của Hiện Tại</v>
       </c>
       <c r="B20" t="str">
         <v>9786045678919</v>
       </c>
       <c r="C20" t="str">
-        <v>NXB Hội Nhà Văn</v>
+        <v>NXB Tổng Hợp TP.HCM</v>
       </c>
       <c r="D20" t="str">
-        <v>Văn học</v>
-      </c>
-      <c r="E20">
-        <v>145000</v>
+        <v>Tâm lý học</v>
+      </c>
+      <c r="E20" t="str">
+        <v>135.000</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Thế Giới Quả Là Rộng Lớn Và Có Nhiều Việc Phải Làm</v>
+        <v>Đắc Nhân Tâm - Bìa Cứng Special</v>
       </c>
       <c r="B21" t="str">
         <v>9786045678920</v>
@@ -750,10 +750,10 @@
         <v>NXB Trẻ</v>
       </c>
       <c r="D21" t="str">
-        <v>Kinh tế</v>
-      </c>
-      <c r="E21">
-        <v>105000</v>
+        <v>Kỹ năng sống</v>
+      </c>
+      <c r="E21" t="str">
+        <v>180.000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement dual-mode integration, bipartite optimal matching, progressive crosswalk, and FAHASA multi-branch support
</commit_message>
<xml_diff>
--- a/sample-data/danh-muc-san-pham-chuan.xlsx
+++ b/sample-data/danh-muc-san-pham-chuan.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,347 +418,177 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Đắc Nhân Tâm</v>
+        <v>Mãi mãi tuổi hai mươi (Độc quyền - Bìa cứng)</v>
       </c>
       <c r="B2" t="str">
-        <v>9786045678901</v>
+        <v>9786042392440</v>
       </c>
       <c r="C2" t="str">
-        <v>NXB Trẻ</v>
+        <v>NXB Kim Đồng</v>
       </c>
       <c r="D2" t="str">
-        <v>Kỹ năng sống</v>
+        <v>Văn học</v>
       </c>
       <c r="E2" t="str">
-        <v>86.000</v>
+        <v>135.000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Nhà Giả Kim</v>
+        <v>Đắc Nhân Tâm</v>
       </c>
       <c r="B3" t="str">
-        <v>9786045678902</v>
+        <v>9786045678901</v>
       </c>
       <c r="C3" t="str">
-        <v>NXB Nhã Nam</v>
+        <v>NXB Trẻ</v>
       </c>
       <c r="D3" t="str">
-        <v>Văn học</v>
+        <v>Kỹ năng sống</v>
       </c>
       <c r="E3" t="str">
-        <v>79.000</v>
+        <v>86.000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Tuổi Trẻ Đáng Giá Bao Nhiêu</v>
+        <v>Nhà Giả Kim</v>
       </c>
       <c r="B4" t="str">
-        <v>9786045678903</v>
+        <v>9786045678902</v>
       </c>
       <c r="C4" t="str">
-        <v>NXB Hội Nhà Văn</v>
+        <v>NXB Nhã Nam</v>
       </c>
       <c r="D4" t="str">
-        <v>Kỹ năng sống</v>
+        <v>Văn học</v>
       </c>
       <c r="E4" t="str">
-        <v>90.000</v>
+        <v>79.000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Cà Phê Cùng Tony</v>
+        <v>Tuổi Trẻ Đáng Giá Bao Nhiêu</v>
       </c>
       <c r="B5" t="str">
-        <v>9786045678904</v>
+        <v>9786045678903</v>
       </c>
       <c r="C5" t="str">
-        <v>NXB Trẻ</v>
+        <v>NXB Hội Nhà Văn</v>
       </c>
       <c r="D5" t="str">
         <v>Kỹ năng sống</v>
       </c>
       <c r="E5" t="str">
-        <v>95.000</v>
+        <v>90.000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Tôi Thấy Hoa Vàng Trên Cỏ Xanh</v>
+        <v>Cà Phê Cùng Tony</v>
       </c>
       <c r="B6" t="str">
-        <v>9786045678905</v>
+        <v>9786045678904</v>
       </c>
       <c r="C6" t="str">
         <v>NXB Trẻ</v>
       </c>
       <c r="D6" t="str">
-        <v>Văn học</v>
+        <v>Kỹ năng sống</v>
       </c>
       <c r="E6" t="str">
-        <v>125.000</v>
+        <v>95.000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Đời Thay Đổi Khi Chúng Ta Thay Đổi</v>
+        <v>Tôi Thấy Hoa Vàng Trên Cỏ Xanh</v>
       </c>
       <c r="B7" t="str">
-        <v>9786045678906</v>
+        <v>9786045678905</v>
       </c>
       <c r="C7" t="str">
         <v>NXB Trẻ</v>
       </c>
       <c r="D7" t="str">
-        <v>Kỹ năng sống</v>
+        <v>Văn học</v>
       </c>
       <c r="E7" t="str">
-        <v>68.000</v>
+        <v>125.000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Cha Giàu Cha Nghèo</v>
+        <v>Dế Mèn Phiêu Lưu Ký</v>
       </c>
       <c r="B8" t="str">
-        <v>9786045678907</v>
+        <v>9786045678913</v>
       </c>
       <c r="C8" t="str">
-        <v>NXB Trẻ</v>
+        <v>NXB Kim Đồng</v>
       </c>
       <c r="D8" t="str">
-        <v>Kinh doanh</v>
+        <v>Thiếu nhi</v>
       </c>
       <c r="E8" t="str">
-        <v>115.000</v>
+        <v>55.000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Đọc Vị Bất Kỳ Ai</v>
+        <v>Số Đỏ</v>
       </c>
       <c r="B9" t="str">
-        <v>9786045678908</v>
+        <v>9786045678910</v>
       </c>
       <c r="C9" t="str">
-        <v>NXB Thế Giới</v>
+        <v>NXB Văn Học</v>
       </c>
       <c r="D9" t="str">
-        <v>Tâm lý học</v>
+        <v>Văn học</v>
       </c>
       <c r="E9" t="str">
-        <v>89.000</v>
+        <v>65.000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Mắt Biếc</v>
+        <v>Tư Duy Nhanh Và Chậm</v>
       </c>
       <c r="B10" t="str">
-        <v>9786045678909</v>
+        <v>9786045678911</v>
       </c>
       <c r="C10" t="str">
-        <v>NXB Trẻ</v>
+        <v>NXB Thế Giới</v>
       </c>
       <c r="D10" t="str">
-        <v>Văn học</v>
+        <v>Tâm lý học</v>
       </c>
       <c r="E10" t="str">
-        <v>110.000</v>
+        <v>210.000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Số Đỏ</v>
+        <v>Hạt Giống Tâm Hồn</v>
       </c>
       <c r="B11" t="str">
-        <v>9786045678910</v>
+        <v>9786045678918</v>
       </c>
       <c r="C11" t="str">
-        <v>NXB Văn Học</v>
+        <v>NXB Tổng Hợp TP.HCM</v>
       </c>
       <c r="D11" t="str">
-        <v>Văn học</v>
+        <v>Tâm lý học</v>
       </c>
       <c r="E11" t="str">
-        <v>65.000</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Tư Duy Nhanh Và Chậm</v>
-      </c>
-      <c r="B12" t="str">
-        <v>9786045678911</v>
-      </c>
-      <c r="C12" t="str">
-        <v>NXB Thế Giới</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Tâm lý học</v>
-      </c>
-      <c r="E12" t="str">
-        <v>210.000</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Khéo Ăn Nói Sẽ Có Được Thiên Hạ</v>
-      </c>
-      <c r="B13" t="str">
-        <v>9786045678912</v>
-      </c>
-      <c r="C13" t="str">
-        <v>NXB Văn Học</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Kỹ năng sống</v>
-      </c>
-      <c r="E13" t="str">
-        <v>118.000</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Dế Mèn Phiêu Lưu Ký</v>
-      </c>
-      <c r="B14" t="str">
-        <v>9786045678913</v>
-      </c>
-      <c r="C14" t="str">
-        <v>NXB Kim Đồng</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Thiếu nhi</v>
-      </c>
-      <c r="E14" t="str">
-        <v>55.000</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Chiếc Thuyền Ngoài Xa</v>
-      </c>
-      <c r="B15" t="str">
-        <v>9786045678914</v>
-      </c>
-      <c r="C15" t="str">
-        <v>NXB Văn Học</v>
-      </c>
-      <c r="D15" t="str">
-        <v>Văn học</v>
-      </c>
-      <c r="E15" t="str">
-        <v>48.000</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Tắt Đèn</v>
-      </c>
-      <c r="B16" t="str">
-        <v>9786045678915</v>
-      </c>
-      <c r="C16" t="str">
-        <v>NXB Văn Học</v>
-      </c>
-      <c r="D16" t="str">
-        <v>Văn học</v>
-      </c>
-      <c r="E16" t="str">
-        <v>52.000</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>Lão Hạc</v>
-      </c>
-      <c r="B17" t="str">
-        <v>9786045678916</v>
-      </c>
-      <c r="C17" t="str">
-        <v>NXB Văn Học</v>
-      </c>
-      <c r="D17" t="str">
-        <v>Văn học</v>
-      </c>
-      <c r="E17" t="str">
-        <v>45.000</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Vợ Nhặt</v>
-      </c>
-      <c r="B18" t="str">
-        <v>9786045678917</v>
-      </c>
-      <c r="C18" t="str">
-        <v>NXB Văn Học</v>
-      </c>
-      <c r="D18" t="str">
-        <v>Văn học</v>
-      </c>
-      <c r="E18" t="str">
-        <v>42.000</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Hạt Giống Tâm Hồn</v>
-      </c>
-      <c r="B19" t="str">
-        <v>9786045678918</v>
-      </c>
-      <c r="C19" t="str">
-        <v>NXB Tổng Hợp TP.HCM</v>
-      </c>
-      <c r="D19" t="str">
-        <v>Tâm lý học</v>
-      </c>
-      <c r="E19" t="str">
         <v>75.000</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Sức Mạnh Của Hiện Tại</v>
-      </c>
-      <c r="B20" t="str">
-        <v>9786045678919</v>
-      </c>
-      <c r="C20" t="str">
-        <v>NXB Tổng Hợp TP.HCM</v>
-      </c>
-      <c r="D20" t="str">
-        <v>Tâm lý học</v>
-      </c>
-      <c r="E20" t="str">
-        <v>135.000</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Đắc Nhân Tâm - Bìa Cứng Special</v>
-      </c>
-      <c r="B21" t="str">
-        <v>9786045678920</v>
-      </c>
-      <c r="C21" t="str">
-        <v>NXB Trẻ</v>
-      </c>
-      <c r="D21" t="str">
-        <v>Kỹ năng sống</v>
-      </c>
-      <c r="E21" t="str">
-        <v>180.000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>